<commit_message>
Added new RDF data schemes and visual schemes, and fixed xlsx-spreadsheets for economy-table14-19
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table14.xlsx
+++ b/sources/table_normalization/xlsx/economy-table14.xlsx
@@ -384,7 +384,6 @@
     <xf numFmtId="165" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -406,6 +405,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -418,7 +419,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal 2" xfId="2"/>
@@ -908,10 +908,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="13" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24">
+      <c r="B1" s="23">
         <v>3</v>
       </c>
     </row>
@@ -920,109 +920,109 @@
       <c r="B2" s="6"/>
     </row>
     <row r="3" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="27"/>
+      <c r="B3" s="26"/>
     </row>
     <row r="4" spans="1:21" ht="13" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="27" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="13" x14ac:dyDescent="0.3">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="28" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="13" x14ac:dyDescent="0.3">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="29" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="13" x14ac:dyDescent="0.3">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="28" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="13" x14ac:dyDescent="0.3">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="30" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="13" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="31" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="13" x14ac:dyDescent="0.3">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="25" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:21" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39"/>
-      <c r="B13" s="35" t="s">
+      <c r="A13" s="34"/>
+      <c r="B13" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="36"/>
-      <c r="D13" s="35" t="s">
+      <c r="C13" s="37"/>
+      <c r="D13" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="E13" s="36"/>
-      <c r="F13" s="35" t="s">
+      <c r="E13" s="37"/>
+      <c r="F13" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="36"/>
-      <c r="H13" s="35" t="s">
+      <c r="G13" s="37"/>
+      <c r="H13" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="36"/>
-      <c r="J13" s="35" t="s">
+      <c r="I13" s="37"/>
+      <c r="J13" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="36"/>
-      <c r="L13" s="35" t="s">
+      <c r="K13" s="37"/>
+      <c r="L13" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="M13" s="36"/>
-      <c r="N13" s="35" t="s">
+      <c r="M13" s="37"/>
+      <c r="N13" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="O13" s="36"/>
-      <c r="P13" s="35" t="s">
+      <c r="O13" s="37"/>
+      <c r="P13" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="Q13" s="36"/>
-      <c r="R13" s="37" t="s">
+      <c r="Q13" s="37"/>
+      <c r="R13" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="S13" s="38"/>
-      <c r="T13" s="35" t="s">
+      <c r="S13" s="39"/>
+      <c r="T13" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="U13" s="36"/>
+      <c r="U13" s="37"/>
     </row>
     <row r="14" spans="1:21" s="1" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A14" s="34" t="s">
+      <c r="A14" s="33" t="s">
         <v>25</v>
       </c>
       <c r="B14" s="7">
@@ -1105,49 +1105,49 @@
       <c r="F15" s="10">
         <v>85544.36</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="17">
         <v>99515.23</v>
       </c>
-      <c r="H15" s="19">
+      <c r="H15" s="18">
         <v>5789.7</v>
       </c>
-      <c r="I15" s="19">
+      <c r="I15" s="18">
         <v>3537.11</v>
       </c>
-      <c r="J15" s="22">
+      <c r="J15" s="21">
         <v>23032.959999999999</v>
       </c>
-      <c r="K15" s="18">
+      <c r="K15" s="17">
         <v>19048.05</v>
       </c>
-      <c r="L15" s="19">
+      <c r="L15" s="18">
         <v>33161.21</v>
       </c>
-      <c r="M15" s="19">
+      <c r="M15" s="18">
         <v>33292.04</v>
       </c>
-      <c r="N15" s="22">
+      <c r="N15" s="21">
         <v>17651.79</v>
       </c>
-      <c r="O15" s="18">
+      <c r="O15" s="17">
         <v>14860.56</v>
       </c>
-      <c r="P15" s="19">
+      <c r="P15" s="18">
         <v>12876.45</v>
       </c>
-      <c r="Q15" s="19">
+      <c r="Q15" s="18">
         <v>14055.99</v>
       </c>
-      <c r="R15" s="22">
+      <c r="R15" s="21">
         <v>14137.53</v>
       </c>
-      <c r="S15" s="18">
+      <c r="S15" s="17">
         <v>11660.7</v>
       </c>
-      <c r="T15" s="22">
+      <c r="T15" s="21">
         <v>213171.28</v>
       </c>
-      <c r="U15" s="18">
+      <c r="U15" s="17">
         <v>222089.19</v>
       </c>
     </row>
@@ -1170,49 +1170,49 @@
       <c r="F16" s="10">
         <v>19359.02</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="17">
         <v>26375.4</v>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="18">
         <v>4069.1</v>
       </c>
-      <c r="I16" s="19">
+      <c r="I16" s="18">
         <v>4036.39</v>
       </c>
-      <c r="J16" s="22">
+      <c r="J16" s="21">
         <v>10109.06</v>
       </c>
-      <c r="K16" s="18">
+      <c r="K16" s="17">
         <v>10458.11</v>
       </c>
-      <c r="L16" s="19">
+      <c r="L16" s="18">
         <v>18296.07</v>
       </c>
-      <c r="M16" s="19">
+      <c r="M16" s="18">
         <v>18209.580000000002</v>
       </c>
-      <c r="N16" s="22">
+      <c r="N16" s="21">
         <v>10885.65</v>
       </c>
-      <c r="O16" s="18">
+      <c r="O16" s="17">
         <v>11036.03</v>
       </c>
-      <c r="P16" s="19">
+      <c r="P16" s="18">
         <v>7631.45</v>
       </c>
-      <c r="Q16" s="19">
+      <c r="Q16" s="18">
         <v>10046.33</v>
       </c>
-      <c r="R16" s="22">
+      <c r="R16" s="21">
         <v>6979.41</v>
       </c>
-      <c r="S16" s="18">
+      <c r="S16" s="17">
         <v>9684.18</v>
       </c>
-      <c r="T16" s="22">
+      <c r="T16" s="21">
         <v>92738.880000000005</v>
       </c>
-      <c r="U16" s="18">
+      <c r="U16" s="17">
         <v>105745.29</v>
       </c>
     </row>
@@ -1235,49 +1235,49 @@
       <c r="F17" s="10">
         <v>33014.82</v>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="17">
         <v>26877.73</v>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="18">
         <v>10990.63</v>
       </c>
-      <c r="I17" s="19">
+      <c r="I17" s="18">
         <v>13631.41</v>
       </c>
-      <c r="J17" s="22">
+      <c r="J17" s="21">
         <v>29436.18</v>
       </c>
-      <c r="K17" s="18">
+      <c r="K17" s="17">
         <v>27713.96</v>
       </c>
-      <c r="L17" s="19">
+      <c r="L17" s="18">
         <v>36550</v>
       </c>
-      <c r="M17" s="19">
+      <c r="M17" s="18">
         <v>45900.13</v>
       </c>
-      <c r="N17" s="22">
+      <c r="N17" s="21">
         <v>24170.07</v>
       </c>
-      <c r="O17" s="18">
+      <c r="O17" s="17">
         <v>25320.14</v>
       </c>
-      <c r="P17" s="19">
+      <c r="P17" s="18">
         <v>23851.89</v>
       </c>
-      <c r="Q17" s="19">
+      <c r="Q17" s="18">
         <v>20438.349999999999</v>
       </c>
-      <c r="R17" s="22">
+      <c r="R17" s="21">
         <v>26214.9</v>
       </c>
-      <c r="S17" s="18">
+      <c r="S17" s="17">
         <v>24471.74</v>
       </c>
-      <c r="T17" s="22">
+      <c r="T17" s="21">
         <v>234578.19</v>
       </c>
-      <c r="U17" s="18">
+      <c r="U17" s="17">
         <v>234695.92</v>
       </c>
     </row>
@@ -1300,49 +1300,49 @@
       <c r="F18" s="10">
         <v>13888.3</v>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="17">
         <v>14087.66</v>
       </c>
-      <c r="H18" s="19">
+      <c r="H18" s="18">
         <v>3183.68</v>
       </c>
-      <c r="I18" s="19">
+      <c r="I18" s="18">
         <v>2481.79</v>
       </c>
-      <c r="J18" s="22">
+      <c r="J18" s="21">
         <v>8139.48</v>
       </c>
-      <c r="K18" s="18">
+      <c r="K18" s="17">
         <v>8982.14</v>
       </c>
-      <c r="L18" s="19">
+      <c r="L18" s="18">
         <v>12719.37</v>
       </c>
-      <c r="M18" s="19">
+      <c r="M18" s="18">
         <v>14833.56</v>
       </c>
-      <c r="N18" s="22">
+      <c r="N18" s="21">
         <v>8912.9</v>
       </c>
-      <c r="O18" s="18">
+      <c r="O18" s="17">
         <v>11207.1</v>
       </c>
-      <c r="P18" s="19">
+      <c r="P18" s="18">
         <v>8716.7099999999991</v>
       </c>
-      <c r="Q18" s="19">
+      <c r="Q18" s="18">
         <v>9453.0400000000009</v>
       </c>
-      <c r="R18" s="22">
+      <c r="R18" s="21">
         <v>5853.61</v>
       </c>
-      <c r="S18" s="18">
+      <c r="S18" s="17">
         <v>7474.3</v>
       </c>
-      <c r="T18" s="22">
+      <c r="T18" s="21">
         <v>82713.850000000006</v>
       </c>
-      <c r="U18" s="18">
+      <c r="U18" s="17">
         <v>81929</v>
       </c>
     </row>
@@ -1365,49 +1365,49 @@
       <c r="F19" s="10">
         <v>1304.5999999999999</v>
       </c>
-      <c r="G19" s="18">
+      <c r="G19" s="17">
         <v>990.32</v>
       </c>
-      <c r="H19" s="19">
+      <c r="H19" s="18">
         <v>55.4</v>
       </c>
-      <c r="I19" s="19">
+      <c r="I19" s="18">
         <v>55.6</v>
       </c>
-      <c r="J19" s="22">
+      <c r="J19" s="21">
         <v>739.36</v>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="17">
         <v>343.72</v>
       </c>
-      <c r="L19" s="19">
+      <c r="L19" s="18">
         <v>323.39999999999998</v>
       </c>
-      <c r="M19" s="19">
+      <c r="M19" s="18">
         <v>181.2</v>
       </c>
-      <c r="N19" s="22">
+      <c r="N19" s="21">
         <v>449.08</v>
       </c>
-      <c r="O19" s="18">
+      <c r="O19" s="17">
         <v>470.36</v>
       </c>
-      <c r="P19" s="19">
+      <c r="P19" s="18">
         <v>183.6</v>
       </c>
-      <c r="Q19" s="19">
+      <c r="Q19" s="18">
         <v>557.44000000000005</v>
       </c>
-      <c r="R19" s="22">
+      <c r="R19" s="21">
         <v>0</v>
       </c>
-      <c r="S19" s="18">
+      <c r="S19" s="17">
         <v>0</v>
       </c>
-      <c r="T19" s="22">
+      <c r="T19" s="21">
         <v>4633.92</v>
       </c>
-      <c r="U19" s="18">
+      <c r="U19" s="17">
         <v>4546.5600000000004</v>
       </c>
     </row>
@@ -1430,49 +1430,49 @@
       <c r="F20" s="10">
         <v>5732.3</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="17">
         <v>6683.82</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="18">
         <v>211.66</v>
       </c>
-      <c r="I20" s="19">
+      <c r="I20" s="18">
         <v>640.67999999999995</v>
       </c>
-      <c r="J20" s="22">
+      <c r="J20" s="21">
         <v>1632.48</v>
       </c>
-      <c r="K20" s="18">
+      <c r="K20" s="17">
         <v>1705.06</v>
       </c>
-      <c r="L20" s="19">
+      <c r="L20" s="18">
         <v>3728.56</v>
       </c>
-      <c r="M20" s="19">
+      <c r="M20" s="18">
         <v>3171.48</v>
       </c>
-      <c r="N20" s="22">
+      <c r="N20" s="21">
         <v>1578.9</v>
       </c>
-      <c r="O20" s="18">
+      <c r="O20" s="17">
         <v>1458.82</v>
       </c>
-      <c r="P20" s="19">
+      <c r="P20" s="18">
         <v>655.88</v>
       </c>
-      <c r="Q20" s="19">
+      <c r="Q20" s="18">
         <v>1039.3</v>
       </c>
-      <c r="R20" s="22">
+      <c r="R20" s="21">
         <v>916.94</v>
       </c>
-      <c r="S20" s="18">
+      <c r="S20" s="17">
         <v>1126.32</v>
       </c>
-      <c r="T20" s="22">
+      <c r="T20" s="21">
         <v>19089.3</v>
       </c>
-      <c r="U20" s="18">
+      <c r="U20" s="17">
         <v>18291.3</v>
       </c>
     </row>
@@ -1495,49 +1495,49 @@
       <c r="F21" s="10">
         <v>74661.72</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="17">
         <v>64648.87</v>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="18">
         <v>4044.96</v>
       </c>
-      <c r="I21" s="19">
+      <c r="I21" s="18">
         <v>4621.8</v>
       </c>
-      <c r="J21" s="22">
+      <c r="J21" s="21">
         <v>18174.63</v>
       </c>
-      <c r="K21" s="18">
+      <c r="K21" s="17">
         <v>18566.400000000001</v>
       </c>
-      <c r="L21" s="19">
+      <c r="L21" s="18">
         <v>39267.67</v>
       </c>
-      <c r="M21" s="19">
+      <c r="M21" s="18">
         <v>32008.68</v>
       </c>
-      <c r="N21" s="22">
+      <c r="N21" s="21">
         <v>22451.24</v>
       </c>
-      <c r="O21" s="18">
+      <c r="O21" s="17">
         <v>21715.31</v>
       </c>
-      <c r="P21" s="19">
+      <c r="P21" s="18">
         <v>11410.92</v>
       </c>
-      <c r="Q21" s="19">
+      <c r="Q21" s="18">
         <v>12425.02</v>
       </c>
-      <c r="R21" s="22">
+      <c r="R21" s="21">
         <v>17019.169999999998</v>
       </c>
-      <c r="S21" s="18">
+      <c r="S21" s="17">
         <v>13080.2</v>
       </c>
-      <c r="T21" s="22">
+      <c r="T21" s="21">
         <v>224645.51</v>
       </c>
-      <c r="U21" s="18">
+      <c r="U21" s="17">
         <v>202056.6</v>
       </c>
     </row>
@@ -1560,49 +1560,49 @@
       <c r="F22" s="10">
         <v>53209.8</v>
       </c>
-      <c r="G22" s="18">
+      <c r="G22" s="17">
         <v>50370.2</v>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="18">
         <v>2456.12</v>
       </c>
-      <c r="I22" s="19">
+      <c r="I22" s="18">
         <v>551</v>
       </c>
-      <c r="J22" s="22">
+      <c r="J22" s="21">
         <v>9407.52</v>
       </c>
-      <c r="K22" s="18">
+      <c r="K22" s="17">
         <v>6214.92</v>
       </c>
-      <c r="L22" s="19">
+      <c r="L22" s="18">
         <v>8022.76</v>
       </c>
-      <c r="M22" s="19">
+      <c r="M22" s="18">
         <v>9786.56</v>
       </c>
-      <c r="N22" s="22">
+      <c r="N22" s="21">
         <v>6884.8</v>
       </c>
-      <c r="O22" s="18">
+      <c r="O22" s="17">
         <v>5000.5200000000004</v>
       </c>
-      <c r="P22" s="19">
+      <c r="P22" s="18">
         <v>4357.6000000000004</v>
       </c>
-      <c r="Q22" s="19">
+      <c r="Q22" s="18">
         <v>3693.28</v>
       </c>
-      <c r="R22" s="22">
+      <c r="R22" s="21">
         <v>3465.64</v>
       </c>
-      <c r="S22" s="18">
+      <c r="S22" s="17">
         <v>2482.2399999999998</v>
       </c>
-      <c r="T22" s="22">
+      <c r="T22" s="21">
         <v>95393.44</v>
       </c>
-      <c r="U22" s="18">
+      <c r="U22" s="17">
         <v>82859.28</v>
       </c>
     </row>
@@ -1625,49 +1625,49 @@
       <c r="F23" s="10">
         <v>67657.47</v>
       </c>
-      <c r="G23" s="18">
+      <c r="G23" s="17">
         <v>71860.399999999994</v>
       </c>
-      <c r="H23" s="19">
+      <c r="H23" s="18">
         <v>5779.68</v>
       </c>
-      <c r="I23" s="19">
+      <c r="I23" s="18">
         <v>5415.05</v>
       </c>
-      <c r="J23" s="22">
+      <c r="J23" s="21">
         <v>24301.05</v>
       </c>
-      <c r="K23" s="18">
+      <c r="K23" s="17">
         <v>24172.26</v>
       </c>
-      <c r="L23" s="19">
+      <c r="L23" s="18">
         <v>57114.65</v>
       </c>
-      <c r="M23" s="19">
+      <c r="M23" s="18">
         <v>56471.76</v>
       </c>
-      <c r="N23" s="22">
+      <c r="N23" s="21">
         <v>18561.900000000001</v>
       </c>
-      <c r="O23" s="18">
+      <c r="O23" s="17">
         <v>22620.36</v>
       </c>
-      <c r="P23" s="19">
+      <c r="P23" s="18">
         <v>18728.330000000002</v>
       </c>
-      <c r="Q23" s="19">
+      <c r="Q23" s="18">
         <v>20505.189999999999</v>
       </c>
-      <c r="R23" s="22">
+      <c r="R23" s="21">
         <v>16676.16</v>
       </c>
-      <c r="S23" s="18">
+      <c r="S23" s="17">
         <v>18933.080000000002</v>
       </c>
-      <c r="T23" s="22">
+      <c r="T23" s="21">
         <v>247218.88</v>
       </c>
-      <c r="U23" s="18">
+      <c r="U23" s="17">
         <v>261329.5</v>
       </c>
     </row>
@@ -1690,49 +1690,49 @@
       <c r="F24" s="10">
         <v>27029.46</v>
       </c>
-      <c r="G24" s="18">
+      <c r="G24" s="17">
         <v>17309.39</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="18">
         <v>1471.93</v>
       </c>
-      <c r="I24" s="19">
+      <c r="I24" s="18">
         <v>582.70000000000005</v>
       </c>
-      <c r="J24" s="22">
+      <c r="J24" s="21">
         <v>3182.52</v>
       </c>
-      <c r="K24" s="18">
+      <c r="K24" s="17">
         <v>2693.71</v>
       </c>
-      <c r="L24" s="19">
+      <c r="L24" s="18">
         <v>8584.08</v>
       </c>
-      <c r="M24" s="19">
+      <c r="M24" s="18">
         <v>8885.9699999999993</v>
       </c>
-      <c r="N24" s="22">
+      <c r="N24" s="21">
         <v>5089.8100000000004</v>
       </c>
-      <c r="O24" s="18">
+      <c r="O24" s="17">
         <v>3617.37</v>
       </c>
-      <c r="P24" s="19">
+      <c r="P24" s="18">
         <v>2101.83</v>
       </c>
-      <c r="Q24" s="19">
+      <c r="Q24" s="18">
         <v>1531.88</v>
       </c>
-      <c r="R24" s="22">
+      <c r="R24" s="21">
         <v>1623.98</v>
       </c>
-      <c r="S24" s="18">
+      <c r="S24" s="17">
         <v>4098.2700000000004</v>
       </c>
-      <c r="T24" s="22">
+      <c r="T24" s="21">
         <v>57192.23</v>
       </c>
-      <c r="U24" s="18">
+      <c r="U24" s="17">
         <v>49547.08</v>
       </c>
     </row>
@@ -1755,49 +1755,49 @@
       <c r="F25" s="10">
         <v>2303.1588018832899</v>
       </c>
-      <c r="G25" s="18">
+      <c r="G25" s="17">
         <v>2290.4898691091198</v>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="18">
         <v>887.75947528178006</v>
       </c>
-      <c r="I25" s="19">
+      <c r="I25" s="18">
         <v>816.934176687177</v>
       </c>
-      <c r="J25" s="22">
+      <c r="J25" s="21">
         <v>2574.7755466356102</v>
       </c>
-      <c r="K25" s="18">
+      <c r="K25" s="17">
         <v>2541.1737714501</v>
       </c>
-      <c r="L25" s="19">
+      <c r="L25" s="18">
         <v>2944.9483963214602</v>
       </c>
-      <c r="M25" s="19">
+      <c r="M25" s="18">
         <v>3106.1449363046299</v>
       </c>
-      <c r="N25" s="22">
+      <c r="N25" s="21">
         <v>1948.2131039549399</v>
       </c>
-      <c r="O25" s="18">
+      <c r="O25" s="17">
         <v>2120.6844910865502</v>
       </c>
-      <c r="P25" s="19">
+      <c r="P25" s="18">
         <v>1686.8220491275599</v>
       </c>
-      <c r="Q25" s="19">
+      <c r="Q25" s="18">
         <v>1787.52677056676</v>
       </c>
-      <c r="R25" s="22">
+      <c r="R25" s="21">
         <v>1885.1343223941301</v>
       </c>
-      <c r="S25" s="18">
+      <c r="S25" s="17">
         <v>1924.4417882334601</v>
       </c>
-      <c r="T25" s="22">
+      <c r="T25" s="21">
         <v>18022.710225611201</v>
       </c>
-      <c r="U25" s="18">
+      <c r="U25" s="17">
         <v>18260.782683245099</v>
       </c>
     </row>
@@ -1820,49 +1820,49 @@
       <c r="F26" s="10">
         <v>4324.38</v>
       </c>
-      <c r="G26" s="18">
+      <c r="G26" s="17">
         <v>4639.54</v>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="18">
         <v>318.92</v>
       </c>
-      <c r="I26" s="19">
+      <c r="I26" s="18">
         <v>414.33</v>
       </c>
-      <c r="J26" s="22">
+      <c r="J26" s="21">
         <v>1597.7950000000001</v>
       </c>
-      <c r="K26" s="18">
+      <c r="K26" s="17">
         <v>1842.875</v>
       </c>
-      <c r="L26" s="19">
+      <c r="L26" s="18">
         <v>1911.86</v>
       </c>
-      <c r="M26" s="19">
+      <c r="M26" s="18">
         <v>2666.145</v>
       </c>
-      <c r="N26" s="22">
+      <c r="N26" s="21">
         <v>823.73500000000001</v>
       </c>
-      <c r="O26" s="18">
+      <c r="O26" s="17">
         <v>1484.2950000000001</v>
       </c>
-      <c r="P26" s="19">
+      <c r="P26" s="18">
         <v>1347.92</v>
       </c>
-      <c r="Q26" s="19">
+      <c r="Q26" s="18">
         <v>1140.53</v>
       </c>
-      <c r="R26" s="22">
+      <c r="R26" s="21">
         <v>1191.4449999999999</v>
       </c>
-      <c r="S26" s="18">
+      <c r="S26" s="17">
         <v>904.53</v>
       </c>
-      <c r="T26" s="22">
+      <c r="T26" s="21">
         <v>17396.900000000001</v>
       </c>
-      <c r="U26" s="18">
+      <c r="U26" s="17">
         <v>17217.849999999999</v>
       </c>
     </row>
@@ -1885,49 +1885,49 @@
       <c r="F27" s="10">
         <v>63758.48</v>
       </c>
-      <c r="G27" s="18">
+      <c r="G27" s="17">
         <v>73017.95</v>
       </c>
-      <c r="H27" s="19">
+      <c r="H27" s="18">
         <v>4903.03</v>
       </c>
-      <c r="I27" s="19">
+      <c r="I27" s="18">
         <v>5822.66</v>
       </c>
-      <c r="J27" s="22">
+      <c r="J27" s="21">
         <v>12698.59</v>
       </c>
-      <c r="K27" s="18">
+      <c r="K27" s="17">
         <v>17444.98</v>
       </c>
-      <c r="L27" s="19">
+      <c r="L27" s="18">
         <v>28863.43</v>
       </c>
-      <c r="M27" s="19">
+      <c r="M27" s="18">
         <v>28772.09</v>
       </c>
-      <c r="N27" s="22">
+      <c r="N27" s="21">
         <v>18800.009999999998</v>
       </c>
-      <c r="O27" s="18">
+      <c r="O27" s="17">
         <v>16936.36</v>
       </c>
-      <c r="P27" s="19">
+      <c r="P27" s="18">
         <v>7784.43</v>
       </c>
-      <c r="Q27" s="19">
+      <c r="Q27" s="18">
         <v>9140.4500000000007</v>
       </c>
-      <c r="R27" s="22">
+      <c r="R27" s="21">
         <v>12036.42</v>
       </c>
-      <c r="S27" s="18">
+      <c r="S27" s="17">
         <v>13994.85</v>
       </c>
-      <c r="T27" s="22">
+      <c r="T27" s="21">
         <v>172585.69</v>
       </c>
-      <c r="U27" s="18">
+      <c r="U27" s="17">
         <v>189158.06</v>
       </c>
     </row>
@@ -1937,84 +1937,84 @@
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
       <c r="F28" s="12"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="20"/>
-      <c r="P28" s="21"/>
-      <c r="Q28" s="21"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="20"/>
-      <c r="T28" s="23"/>
-      <c r="U28" s="20"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="20"/>
+      <c r="M28" s="20"/>
+      <c r="N28" s="22"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="20"/>
+      <c r="Q28" s="20"/>
+      <c r="R28" s="22"/>
+      <c r="S28" s="19"/>
+      <c r="T28" s="22"/>
+      <c r="U28" s="19"/>
     </row>
     <row r="29" spans="1:21" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="16">
+      <c r="B29" s="15">
         <v>87842.860384892905</v>
       </c>
-      <c r="C29" s="17">
+      <c r="C29" s="16">
         <v>85406.061560334507</v>
       </c>
-      <c r="D29" s="16">
+      <c r="D29" s="15">
         <v>138251.413145119</v>
       </c>
-      <c r="E29" s="17">
+      <c r="E29" s="16">
         <v>133419.72531947299</v>
       </c>
-      <c r="F29" s="16">
+      <c r="F29" s="15">
         <v>451787.86880188301</v>
       </c>
-      <c r="G29" s="17">
+      <c r="G29" s="16">
         <v>458666.99986910901</v>
       </c>
-      <c r="H29" s="16">
+      <c r="H29" s="15">
         <v>44162.569475281802</v>
       </c>
-      <c r="I29" s="17">
+      <c r="I29" s="16">
         <v>42607.454176687199</v>
       </c>
-      <c r="J29" s="16">
+      <c r="J29" s="15">
         <v>145026.400546636</v>
       </c>
-      <c r="K29" s="17">
+      <c r="K29" s="16">
         <v>141727.35877145</v>
       </c>
-      <c r="L29" s="16">
+      <c r="L29" s="15">
         <v>251488.00839632101</v>
       </c>
-      <c r="M29" s="17">
+      <c r="M29" s="16">
         <v>257285.33993630501</v>
       </c>
-      <c r="N29" s="16">
+      <c r="N29" s="15">
         <v>138208.09810395501</v>
       </c>
-      <c r="O29" s="17">
+      <c r="O29" s="16">
         <v>137847.90949108699</v>
       </c>
-      <c r="P29" s="16">
+      <c r="P29" s="15">
         <v>101333.832049128</v>
       </c>
-      <c r="Q29" s="17">
+      <c r="Q29" s="16">
         <v>105814.326770567</v>
       </c>
-      <c r="R29" s="16">
+      <c r="R29" s="15">
         <v>108000.33932239399</v>
       </c>
-      <c r="S29" s="17">
+      <c r="S29" s="16">
         <v>109834.85178823301</v>
       </c>
-      <c r="T29" s="16">
+      <c r="T29" s="15">
         <v>1479380.7802256099</v>
       </c>
-      <c r="U29" s="17">
+      <c r="U29" s="16">
         <v>1487726.4126832499</v>
       </c>
     </row>

</xml_diff>